<commit_message>
Add business-insight layer: exec summary + cedentes/sacados; Codex output brief
- scripts/build_industria_fidc_deck.py: add Executive Summary slide (market
  doubled, independents dominate management, Itau 4-5x behind BTG/QI in
  administration, credit tied to payments) and Cedentes & Sacados slide/sheet
  (named parties by materiality from reports/fidc_clean_named_parties).
- reports/insights_industria_fidc.md: committee-ready market read (who grew/fell,
  Oliveira Trust/QI Tech/BTG stories, cedentes/sacados, Itau competitive gap).
- docs/brief_codex_output.md: brief to reorient Codex from empty infrastructure
  to business-insight output (lead with findings, materialize data not scaffolding,
  fill the thin cedente/sacado layer first).
</commit_message>
<xml_diff>
--- a/outputs/Industria_FIDC_2026-05.xlsx
+++ b/outputs/Industria_FIDC_2026-05.xlsx
@@ -20,7 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotistas" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento Investidor" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emissoes" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cedentes e Sacados" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +58,11 @@
       <i val="1"/>
       <color rgb="008A94A6"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F2A44"/>
     </font>
   </fonts>
   <fills count="3">
@@ -98,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -122,6 +128,7 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2768,7 +2775,461 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cedentes e sacados relevantes (leitura de regulamentos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Maiores CEDENTES (originadores)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Parte</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Setor</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t># Fundos</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Materialidade (R$ bi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Banco BTG Pactual S.A</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Meios de Pagamento e Cartões</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>15.92</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MULTIPLIKE CONSULTORIA E COBRANÇA LTDA</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PJ</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>PagueVeloz Instituição de Pagamento Ltda</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Sem oferta CVM mapeada</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2.01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Banco Bradesco S.A</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Meios de Pagamento e Cartões</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>1.67</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Banco BMG S.A</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PF</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>BRB - BANCO DE BRASÍLIA S.A</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PF</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>UPL DO BRASIL INDÚSTRIA E COMÉRCIO DE INSUMOS AGROPECUÁRIOS S.A</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Agro</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Banco Votorantim S.A</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Sem oferta CVM mapeada</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Serviços Técnicos de Seguro Ltda</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Sem oferta CVM mapeada</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>IBM BRASIL - INDÚSTRIA, MÁQUINAS, E SERVIÇOS LTDA</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PF</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Maiores SACADOS (devedores)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Parte</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Setor</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t># Fundos</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Materialidade (R$ bi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>MERCADO PAGO INSTITUIÇÃO DE PAGAMENTO LTDA</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Meios de Pagamento e Cartões</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Boletos Banco Votorantim S.A</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Sem oferta CVM mapeada</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PJ</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Oliveira Trust Distribuidora de Títulos e Valores Mobiliários S.A</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PJ</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>SafraPay Instituição de Pagamento Ltda</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PJ</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>LAVORO AGRO HOLDING S.A</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Agro</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Latasa Industria e Comercio Ltda</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PF</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>io de Metais Ltda</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Crédito PF</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>MEUCASHCARD SERVIÇOS TECNOLÓGICOS E FINANCEIROS S/A</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Imobiliário</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Rotam do Brasil Agroquímica e Produtos Agrícolas Ltda</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Agro</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Fonte: Toma Conta FIDCs — leitura de regulamentos (cedentes/sacados nomeados, materialidade por PL de fundo). Base: reports/fidc_clean_named_parties.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A29:H29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2923,6 +3384,30 @@
       <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Toma Conta FIDCs — variação anual de PL (ex-FIC) e captação líquida (dimensão mensal). Métrica preferida: variação de PL. Validação de magnitude: ANBIMA (imprensa, 2024). NÃO é o campo 'emissões encerradas'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>partes</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Toma Conta FIDCs — leitura de regulamentos (cedentes/sacados nomeados, materialidade por PL de fundo). Base: reports/fidc_clean_named_parties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>sumario</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Síntese das dimensões do Toma Conta (gestor/admin/custodiante/segmento) consolidadas por conglomerado.</t>
         </is>
       </c>
     </row>

</xml_diff>